<commit_message>
Made this pice of shit run but with only one address
</commit_message>
<xml_diff>
--- a/debian/old/четец(1)/четец/output.xlsx
+++ b/debian/old/четец(1)/четец/output.xlsx
@@ -13,6 +13,7 @@
     <sheet name="09-09-2025" sheetId="8" r:id="rId8"/>
     <sheet name="10-09-2025" sheetId="9" r:id="rId9"/>
     <sheet name="11-09-2025" sheetId="10" r:id="rId10"/>
+    <sheet name="21-09-2025" sheetId="11" r:id="rId11"/>
   </sheets>
 </workbook>
 </file>
@@ -7240,6 +7241,123 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:Q2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Date</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Time</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Meter Name</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Active Energy</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Voltage L1</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Voltage L2</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Voltage L3</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Current L1</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Current L2</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Current L3</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Active power L1</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Active power L2</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Active power L3</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Power factor L1</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Power factor L2</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Power factor L3</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Total active power</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>21.09.2025 г.</v>
+      </c>
+      <c r="B2" t="str">
+        <v>10:53:59 ч.</v>
+      </c>
+      <c r="C2" t="str">
+        <v>TBA-8</v>
+      </c>
+      <c r="D2">
+        <v>152140.11790587843</v>
+      </c>
+      <c r="E2">
+        <v>234.4932861328125</v>
+      </c>
+      <c r="F2">
+        <v>235.07278442382812</v>
+      </c>
+      <c r="G2">
+        <v>236.4445037841797</v>
+      </c>
+      <c r="H2">
+        <v>1.4569017887115479</v>
+      </c>
+      <c r="I2">
+        <v>1.5329453945159912</v>
+      </c>
+      <c r="J2">
+        <v>1.4757840633392334</v>
+      </c>
+      <c r="K2">
+        <v>265.0392761230469</v>
+      </c>
+      <c r="L2">
+        <v>213.35438537597656</v>
+      </c>
+      <c r="M2">
+        <v>210.8924560546875</v>
+      </c>
+      <c r="N2">
+        <v>0.7760823965072632</v>
+      </c>
+      <c r="O2">
+        <v>0.5922360420227051</v>
+      </c>
+      <c r="P2">
+        <v>0.6025905013084412</v>
+      </c>
+      <c r="Q2">
+        <v>683.976318359375</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H241"/>

</xml_diff>